<commit_message>
Complete Stage 1 with twelve encoders and GTEx, and record the Stage 2 decision
Stage1_analysis.ipynb now runs twelve frozen encoders, four per modality,
on the mRNA stability pilot and on a GTEx pilot built by
Code/build_gtex_pilot.py, with result notes and interpretations after
every output. The run adds PCA variance bands, attention permutation
nulls, and published-split comparisons with BioLangFusion and IsoFormer.

The README, docs, project notes, October 7 slides, research canvas, and
Gantt plan describe the current results and the Stage 2 alignment
decision, which lives in the notes and the Overleaf project.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016z8BM931pKqvCtYb6578dV
</commit_message>
<xml_diff>
--- a/docs/Research_Project_Plan_Gantt.xlsx
+++ b/docs/Research_Project_Plan_Gantt.xlsx
@@ -13,7 +13,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -63,12 +63,12 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="FF486A86"/>
+      <color rgb="FF202A33"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="FF486A86"/>
+      <color rgb="FF202A33"/>
       <sz val="11"/>
     </font>
     <font>
@@ -79,6 +79,11 @@
     <font>
       <name val="Arial"/>
       <color rgb="FF77558E"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF202A33"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -131,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -238,6 +243,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -580,7 +588,7 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>As of September 29, 2026. Fall weeks start Monday; January–March 2027 is an adjustable monthly horizon.</t>
+          <t>As of October 3, 2026. Fall weeks start Monday; January–March 2027 is an adjustable monthly horizon.</t>
         </is>
       </c>
     </row>
@@ -755,7 +763,7 @@
     <row r="7" ht="29" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Stage 1: understanding and reproducibility</t>
+          <t>Stages 1 and 2: representation analysis and defining alignment</t>
         </is>
       </c>
     </row>
@@ -838,7 +846,7 @@
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>Oct 5</t>
+          <t>Oct 7</t>
         </is>
       </c>
       <c r="F9" s="13" t="str"/>
@@ -896,7 +904,7 @@
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>Oct 4</t>
+          <t>Oct 7</t>
         </is>
       </c>
       <c r="F10" s="13" t="str"/>
@@ -911,7 +919,11 @@
           <t>██</t>
         </is>
       </c>
-      <c r="J10" s="13" t="str"/>
+      <c r="J10" s="22" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="K10" s="13" t="str"/>
       <c r="L10" s="13" t="str"/>
       <c r="M10" s="13" t="str"/>
@@ -938,9 +950,9 @@
           <t>Check train/test separation and preprocessing</t>
         </is>
       </c>
-      <c r="C11" s="21" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="D11" s="15" t="inlineStr">
@@ -950,17 +962,17 @@
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>Oct 4</t>
+          <t>Oct 3</t>
         </is>
       </c>
       <c r="F11" s="13" t="str"/>
       <c r="G11" s="13" t="str"/>
-      <c r="H11" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="I11" s="23" t="inlineStr">
+      <c r="H11" s="19" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="I11" s="19" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -992,9 +1004,9 @@
           <t>Trace runs, seeds and reproducibility evidence</t>
         </is>
       </c>
-      <c r="C12" s="21" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="D12" s="15" t="inlineStr">
@@ -1004,17 +1016,17 @@
       </c>
       <c r="E12" s="15" t="inlineStr">
         <is>
-          <t>Oct 4</t>
+          <t>Oct 3</t>
         </is>
       </c>
       <c r="F12" s="13" t="str"/>
       <c r="G12" s="13" t="str"/>
-      <c r="H12" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="I12" s="23" t="inlineStr">
+      <c r="H12" s="19" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="I12" s="19" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -1046,9 +1058,9 @@
           <t>Interpret representation metrics and pilot findings</t>
         </is>
       </c>
-      <c r="C13" s="21" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="D13" s="15" t="inlineStr">
@@ -1058,17 +1070,17 @@
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>Oct 4</t>
+          <t>Oct 3</t>
         </is>
       </c>
       <c r="F13" s="13" t="str"/>
       <c r="G13" s="13" t="str"/>
-      <c r="H13" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="I13" s="23" t="inlineStr">
+      <c r="H13" s="19" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="I13" s="19" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -1112,7 +1124,7 @@
       </c>
       <c r="E14" s="15" t="inlineStr">
         <is>
-          <t>Oct 4</t>
+          <t>Oct 7</t>
         </is>
       </c>
       <c r="F14" s="13" t="str"/>
@@ -1127,7 +1139,11 @@
           <t>██</t>
         </is>
       </c>
-      <c r="J14" s="13" t="str"/>
+      <c r="J14" s="22" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="K14" s="13" t="str"/>
       <c r="L14" s="13" t="str"/>
       <c r="M14" s="13" t="str"/>
@@ -1154,9 +1170,9 @@
           <t>Map BioLangFusion and IsoFormer inputs, including DNA</t>
         </is>
       </c>
-      <c r="C15" s="25" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="D15" s="15" t="inlineStr">
@@ -1166,13 +1182,13 @@
       </c>
       <c r="E15" s="15" t="inlineStr">
         <is>
-          <t>Sep 30</t>
+          <t>Oct 2</t>
         </is>
       </c>
       <c r="F15" s="13" t="str"/>
       <c r="G15" s="13" t="str"/>
       <c r="H15" s="13" t="str"/>
-      <c r="I15" s="27" t="inlineStr">
+      <c r="I15" s="19" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -1201,12 +1217,12 @@
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>Build and check a BioLangFusion methods pilot</t>
-        </is>
-      </c>
-      <c r="C16" s="25" t="inlineStr">
-        <is>
-          <t>Planned</t>
+          <t>Run published-split comparisons for both datasets</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
       <c r="D16" s="15" t="inlineStr">
@@ -1216,13 +1232,13 @@
       </c>
       <c r="E16" s="15" t="inlineStr">
         <is>
-          <t>Oct 4</t>
+          <t>Oct 3</t>
         </is>
       </c>
       <c r="F16" s="13" t="str"/>
       <c r="G16" s="13" t="str"/>
       <c r="H16" s="13" t="str"/>
-      <c r="I16" s="27" t="inlineStr">
+      <c r="I16" s="19" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -1266,7 +1282,7 @@
       </c>
       <c r="E17" s="15" t="inlineStr">
         <is>
-          <t>Oct 4</t>
+          <t>Oct 7</t>
         </is>
       </c>
       <c r="F17" s="13" t="str"/>
@@ -1281,7 +1297,11 @@
           <t>██</t>
         </is>
       </c>
-      <c r="J17" s="13" t="str"/>
+      <c r="J17" s="22" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="K17" s="13" t="str"/>
       <c r="L17" s="13" t="str"/>
       <c r="M17" s="13" t="str"/>
@@ -1308,7 +1328,7 @@
           <t>Clarify the lab tokenizer and benchmark opportunity</t>
         </is>
       </c>
-      <c r="C18" s="25" t="inlineStr">
+      <c r="C18" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1326,12 +1346,12 @@
       <c r="F18" s="13" t="str"/>
       <c r="G18" s="13" t="str"/>
       <c r="H18" s="13" t="str"/>
-      <c r="I18" s="27" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="J18" s="27" t="inlineStr">
+      <c r="I18" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="J18" s="37" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -1359,12 +1379,12 @@
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>Prepare the Oct 5 evidence and question set</t>
-        </is>
-      </c>
-      <c r="C19" s="25" t="inlineStr">
-        <is>
-          <t>Planned</t>
+          <t>Prepare the Oct 7 evidence and question set</t>
+        </is>
+      </c>
+      <c r="C19" s="21" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="D19" s="15" t="inlineStr">
@@ -1374,18 +1394,22 @@
       </c>
       <c r="E19" s="15" t="inlineStr">
         <is>
-          <t>Oct 4</t>
+          <t>Oct 6</t>
         </is>
       </c>
       <c r="F19" s="13" t="str"/>
       <c r="G19" s="13" t="str"/>
       <c r="H19" s="13" t="str"/>
-      <c r="I19" s="27" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="J19" s="13" t="str"/>
+      <c r="I19" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="J19" s="22" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="K19" s="13" t="str"/>
       <c r="L19" s="13" t="str"/>
       <c r="M19" s="13" t="str"/>
@@ -1409,29 +1433,29 @@
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>Oct 5 review and working alignment definition</t>
-        </is>
-      </c>
-      <c r="C20" s="25" t="inlineStr">
+          <t>Oct 7 review and working alignment definition</t>
+        </is>
+      </c>
+      <c r="C20" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>Oct 5</t>
+          <t>Oct 7</t>
         </is>
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>Oct 5</t>
+          <t>Oct 7</t>
         </is>
       </c>
       <c r="F20" s="13" t="str"/>
       <c r="G20" s="13" t="str"/>
       <c r="H20" s="13" t="str"/>
       <c r="I20" s="13" t="str"/>
-      <c r="J20" s="27" t="inlineStr">
+      <c r="J20" s="37" t="inlineStr">
         <is>
           <t>◆</t>
         </is>
@@ -1462,14 +1486,14 @@
           <t>Revise Stage 1 claims, figures and methods</t>
         </is>
       </c>
-      <c r="C21" s="25" t="inlineStr">
+      <c r="C21" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>Oct 6</t>
+          <t>Oct 8</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
@@ -1481,7 +1505,7 @@
       <c r="G21" s="13" t="str"/>
       <c r="H21" s="13" t="str"/>
       <c r="I21" s="13" t="str"/>
-      <c r="J21" s="27" t="inlineStr">
+      <c r="J21" s="37" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -1512,14 +1536,14 @@
           <t>Specify the first matched comparison protocol</t>
         </is>
       </c>
-      <c r="C22" s="25" t="inlineStr">
+      <c r="C22" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
       <c r="D22" s="15" t="inlineStr">
         <is>
-          <t>Oct 6</t>
+          <t>Oct 8</t>
         </is>
       </c>
       <c r="E22" s="15" t="inlineStr">
@@ -1531,7 +1555,7 @@
       <c r="G22" s="13" t="str"/>
       <c r="H22" s="13" t="str"/>
       <c r="I22" s="13" t="str"/>
-      <c r="J22" s="27" t="inlineStr">
+      <c r="J22" s="37" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -1556,7 +1580,7 @@
     <row r="23" ht="29" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Stage 2: experiments and interpretation</t>
+          <t>Stages 3 and 4: fusion experiments and evaluation</t>
         </is>
       </c>
     </row>
@@ -1569,7 +1593,7 @@
           <t>Harden single-model and simple-fusion baselines</t>
         </is>
       </c>
-      <c r="C24" s="25" t="inlineStr">
+      <c r="C24" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1588,7 +1612,7 @@
       <c r="G24" s="13" t="str"/>
       <c r="H24" s="13" t="str"/>
       <c r="I24" s="13" t="str"/>
-      <c r="J24" s="27" t="inlineStr">
+      <c r="J24" s="37" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -1619,7 +1643,7 @@
           <t>Run matched BioLangFusion-style comparisons</t>
         </is>
       </c>
-      <c r="C25" s="25" t="inlineStr">
+      <c r="C25" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1639,7 +1663,7 @@
       <c r="H25" s="13" t="str"/>
       <c r="I25" s="13" t="str"/>
       <c r="J25" s="13" t="str"/>
-      <c r="K25" s="27" t="inlineStr">
+      <c r="K25" s="37" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -1669,7 +1693,7 @@
           <t>Repeat diagnostics and null/control comparisons</t>
         </is>
       </c>
-      <c r="C26" s="25" t="inlineStr">
+      <c r="C26" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1689,7 +1713,7 @@
       <c r="H26" s="13" t="str"/>
       <c r="I26" s="13" t="str"/>
       <c r="J26" s="13" t="str"/>
-      <c r="K26" s="27" t="inlineStr">
+      <c r="K26" s="37" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -1719,7 +1743,7 @@
           <t>Interpret baseline findings and revise the next experiment</t>
         </is>
       </c>
-      <c r="C27" s="25" t="inlineStr">
+      <c r="C27" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1740,7 +1764,7 @@
       <c r="I27" s="13" t="str"/>
       <c r="J27" s="13" t="str"/>
       <c r="K27" s="13" t="str"/>
-      <c r="L27" s="27" t="inlineStr">
+      <c r="L27" s="37" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -1769,7 +1793,7 @@
           <t>Prepare Coupled Mamba inputs and feasibility tests</t>
         </is>
       </c>
-      <c r="C28" s="25" t="inlineStr">
+      <c r="C28" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1789,12 +1813,12 @@
       <c r="H28" s="13" t="str"/>
       <c r="I28" s="13" t="str"/>
       <c r="J28" s="13" t="str"/>
-      <c r="K28" s="27" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="L28" s="27" t="inlineStr">
+      <c r="K28" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="L28" s="37" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -1823,7 +1847,7 @@
           <t>Evaluate Coupled Mamba against matched baselines</t>
         </is>
       </c>
-      <c r="C29" s="25" t="inlineStr">
+      <c r="C29" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1845,12 +1869,12 @@
       <c r="J29" s="13" t="str"/>
       <c r="K29" s="13" t="str"/>
       <c r="L29" s="13" t="str"/>
-      <c r="M29" s="27" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="N29" s="27" t="inlineStr">
+      <c r="M29" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="N29" s="37" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -2189,7 +2213,7 @@
           <t>Repeat runs, quantify uncertainty and revise claims</t>
         </is>
       </c>
-      <c r="C36" s="25" t="inlineStr">
+      <c r="C36" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -2209,32 +2233,32 @@
       <c r="H36" s="13" t="str"/>
       <c r="I36" s="13" t="str"/>
       <c r="J36" s="13" t="str"/>
-      <c r="K36" s="27" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="L36" s="27" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="M36" s="27" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="N36" s="27" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="O36" s="27" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="P36" s="27" t="inlineStr">
+      <c r="K36" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="L36" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="M36" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="N36" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="O36" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="P36" s="37" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -2259,7 +2283,7 @@
           <t>Synthesize evidence, limitations and next decisions</t>
         </is>
       </c>
-      <c r="C37" s="25" t="inlineStr">
+      <c r="C37" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -2284,12 +2308,12 @@
       <c r="M37" s="13" t="str"/>
       <c r="N37" s="13" t="str"/>
       <c r="O37" s="13" t="str"/>
-      <c r="P37" s="27" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Q37" s="27" t="inlineStr">
+      <c r="P37" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Q37" s="37" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -2617,7 +2641,7 @@
           <t>Prepare final course report, presentation and video</t>
         </is>
       </c>
-      <c r="C43" s="25" t="inlineStr">
+      <c r="C43" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -2642,17 +2666,17 @@
       <c r="M43" s="13" t="str"/>
       <c r="N43" s="13" t="str"/>
       <c r="O43" s="13" t="str"/>
-      <c r="P43" s="27" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Q43" s="27" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="R43" s="27" t="inlineStr">
+      <c r="P43" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Q43" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="R43" s="37" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -2675,7 +2699,7 @@
           <t>Course rehearsal checkpoint</t>
         </is>
       </c>
-      <c r="C44" s="25" t="inlineStr">
+      <c r="C44" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -2702,7 +2726,7 @@
       <c r="O44" s="13" t="str"/>
       <c r="P44" s="13" t="str"/>
       <c r="Q44" s="13" t="str"/>
-      <c r="R44" s="27" t="inlineStr">
+      <c r="R44" s="37" t="inlineStr">
         <is>
           <t>◆</t>
         </is>
@@ -2725,7 +2749,7 @@
           <t>Final course report checkpoint</t>
         </is>
       </c>
-      <c r="C45" s="25" t="inlineStr">
+      <c r="C45" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -2753,7 +2777,7 @@
       <c r="P45" s="13" t="str"/>
       <c r="Q45" s="13" t="str"/>
       <c r="R45" s="13" t="str"/>
-      <c r="S45" s="27" t="inlineStr">
+      <c r="S45" s="37" t="inlineStr">
         <is>
           <t>◆</t>
         </is>
@@ -2775,7 +2799,7 @@
           <t>Course presentation and video checkpoint</t>
         </is>
       </c>
-      <c r="C46" s="25" t="inlineStr">
+      <c r="C46" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -2803,7 +2827,7 @@
       <c r="P46" s="13" t="str"/>
       <c r="Q46" s="13" t="str"/>
       <c r="R46" s="13" t="str"/>
-      <c r="S46" s="27" t="inlineStr">
+      <c r="S46" s="37" t="inlineStr">
         <is>
           <t>◆</t>
         </is>
@@ -2886,7 +2910,7 @@
           <t>Consolidate manuscript and review publication readiness</t>
         </is>
       </c>
-      <c r="C49" s="25" t="inlineStr">
+      <c r="C49" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -2920,12 +2944,12 @@
       <c r="V49" s="13" t="str"/>
       <c r="W49" s="11" t="n"/>
       <c r="X49" s="13" t="str"/>
-      <c r="Y49" s="27" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Z49" s="27" t="inlineStr">
+      <c r="Y49" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Z49" s="37" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -2940,7 +2964,7 @@
           <t>March research review and next-step decision</t>
         </is>
       </c>
-      <c r="C50" s="25" t="inlineStr">
+      <c r="C50" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -2975,7 +2999,7 @@
       <c r="W50" s="11" t="n"/>
       <c r="X50" s="13" t="str"/>
       <c r="Y50" s="13" t="str"/>
-      <c r="Z50" s="27" t="inlineStr">
+      <c r="Z50" s="37" t="inlineStr">
         <is>
           <t>◆</t>
         </is>
@@ -3188,7 +3212,7 @@
     <row r="6" ht="29" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Stage 1: understanding and reproducibility</t>
+          <t>Stages 1 and 2: representation analysis and defining alignment</t>
         </is>
       </c>
     </row>
@@ -3343,7 +3367,7 @@
       </c>
       <c r="C14" s="36" t="inlineStr">
         <is>
-          <t>Compare paper and local checkpoints, tokenization, sequence regions, codon mapping, pooling, labels, splits and metrics for BioLangFusion (CodonBERT stability data) and IsoFormer (GTEx data with genomic DNA). Document how DNA, RNA and protein encoders enter each dataset and the changes needed to adapt the methods.</t>
+          <t>Compare paper and local checkpoints, tokenization, sequence regions, codon mapping, pooling, labels, splits and metrics for BioLangFusion (CodonBERT stability data) and IsoFormer (GTEx data with genomic DNA). Done October 2: the GTEx pilot (2,000 transcripts with 6,000-nucleotide DNA windows) and its registry entry give each encoder its own input.</t>
         </is>
       </c>
       <c r="D14" s="13" t="inlineStr">
@@ -3358,12 +3382,12 @@
       </c>
       <c r="B15" s="36" t="inlineStr">
         <is>
-          <t>Build and check a BioLangFusion methods pilot</t>
+          <t>Run published-split comparisons for both datasets</t>
         </is>
       </c>
       <c r="C15" s="36" t="inlineStr">
         <is>
-          <t>Test input/feature correspondence and selected simple fusion methods in a small prototype. Compare outputs with controls and bring feasibility findings and deviations from the paper to the October 5 review.</t>
+          <t>Done October 3 in Stage1_analysis.ipynb: probes fit on rows sampled from BioLangFusion's published stability split and IsoFormer's GTEx split, scored on their test splits, with each paper's encoder combinations. Trained fusion heads remain Stage 3 work.</t>
         </is>
       </c>
       <c r="D15" s="13" t="inlineStr">
@@ -3418,7 +3442,7 @@
       </c>
       <c r="B18" s="36" t="inlineStr">
         <is>
-          <t>Prepare the Oct 5 evidence and question set</t>
+          <t>Prepare the Oct 7 evidence and question set</t>
         </is>
       </c>
       <c r="C18" s="36" t="inlineStr">
@@ -3438,7 +3462,7 @@
       </c>
       <c r="B19" s="36" t="inlineStr">
         <is>
-          <t>Oct 5 review and working alignment definition</t>
+          <t>Oct 7 review and working alignment definition</t>
         </is>
       </c>
       <c r="C19" s="36" t="inlineStr">
@@ -3495,7 +3519,7 @@
     <row r="22" ht="29" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>Stage 2: experiments and interpretation</t>
+          <t>Stages 3 and 4: fusion experiments and evaluation</t>
         </is>
       </c>
     </row>
@@ -3630,7 +3654,7 @@
       </c>
       <c r="C29" s="36" t="inlineStr">
         <is>
-          <t>After choosing the relevant encoder/layer question, compare selected representations or variance subspaces. Fit any reduction within training data and separate using an earlier layer from truncating or retraining a model.</t>
+          <t>After choosing the relevant encoder/layer question, compare selected representations or variance subspaces. Fit any reduction within training data and separate using an earlier layer from truncating or retraining a model. The representation-level comparison of top-10 principal components and the rest is complete in Stage 1.</t>
         </is>
       </c>
       <c r="D29" s="13" t="inlineStr">
@@ -3670,7 +3694,7 @@
       </c>
       <c r="C31" s="36" t="inlineStr">
         <is>
-          <t>If selected, compare several checkpoints per modality and their combinations, including pairs within one modality, while controlling downstream capacity, input coverage and tuning. Different pretraining corpora alone do not establish complementarity.</t>
+          <t>If selected, compare several checkpoints per modality and their combinations, including pairs within one modality, while controlling downstream capacity, input coverage and tuning. Different pretraining corpora alone do not establish complementarity. Stage 1 already covers twelve encoders, four per modality, at the representation level.</t>
         </is>
       </c>
       <c r="D31" s="13" t="inlineStr">
@@ -4023,14 +4047,14 @@
     <row r="53" ht="42" customHeight="1">
       <c r="A53" s="33" t="inlineStr">
         <is>
-          <t>The team completed the initial six-paper review by September 21. Continued interpretation and discussion run through the October 5 meeting. September 21 start dates for current work are approximate planning anchors.</t>
+          <t>The team completed the initial six-paper review by September 21. Continued interpretation and discussion run through the October 7 meeting. September 21 start dates for current work are approximate planning anchors.</t>
         </is>
       </c>
     </row>
     <row r="54" ht="42" customHeight="1">
       <c r="A54" s="33" t="inlineStr">
         <is>
-          <t>October 5 is the review with Mina and the target for a working alignment definition. Stage 1 includes the immediate revisions after that meeting. Future experiment dates are proposed windows.</t>
+          <t>October 7 is the review with Mina and the target for a working alignment definition. Stage 1 includes the immediate revisions after that meeting. Future experiment dates are proposed windows.</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4075,7 @@
     <row r="57" ht="42" customHeight="1">
       <c r="A57" s="33" t="inlineStr">
         <is>
-          <t>AI supports implementation, paper discussion, analysis and writing throughout the project. Each research task includes interpreting its evidence and revising the resulting claims. OpenAI Codex organized the original plan; Claude assisted with the September 29 revision adding the DNA modality.</t>
+          <t>AI supports implementation, paper discussion, analysis and writing throughout the project. Each research task includes interpreting its evidence and revising the resulting claims. OpenAI Codex organized the original plan; Claude assisted with the September 29 revision adding the DNA modality and the October 3 status update.</t>
         </is>
       </c>
     </row>
@@ -4113,8 +4137,8 @@
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A56:D56"/>
     <mergeCell ref="A37:D37"/>
-    <mergeCell ref="A56:D56"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A22:D22"/>
     <mergeCell ref="A53:D53"/>

</xml_diff>